<commit_message>
Update portfolio components and excel sheet
</commit_message>
<xml_diff>
--- a/public/8 - ANNEXE VI.1 - EPREUVE E5 TABLEAU DE SYNTHESE - BTS SIO 2026 MOUHOUBI Noam.xlsx
+++ b/public/8 - ANNEXE VI.1 - EPREUVE E5 TABLEAU DE SYNTHESE - BTS SIO 2026 MOUHOUBI Noam.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\noamm\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9953DF28-2799-4C1D-846B-CAFCF2A4C787}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4440D4AD-8EE8-47A6-A57C-3FD715E3783D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="46">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -63,9 +63,6 @@
   </si>
   <si>
     <t>▢ SLAM</t>
-  </si>
-  <si>
-    <t>Adresse URL du portfolio :</t>
   </si>
   <si>
     <t>Compétences mises en œuvre
@@ -190,6 +187,15 @@
   </si>
   <si>
     <t>s</t>
+  </si>
+  <si>
+    <t>Adresse URL du portfolio : https://nmouhoubi.com/</t>
+  </si>
+  <si>
+    <t>2024-2026</t>
+  </si>
+  <si>
+    <t>2025-2026</t>
   </si>
 </sst>
 </file>
@@ -199,7 +205,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -263,8 +269,14 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="10"/>
       <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -680,7 +692,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -745,84 +757,99 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="14" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1143,56 +1170,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24" t="s">
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="24"/>
+      <c r="H1" s="28"/>
     </row>
     <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="28"/>
     </row>
     <row r="3" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="B3" s="26"/>
-      <c r="C3" s="26"/>
-      <c r="D3" s="26"/>
-      <c r="E3" s="27"/>
-      <c r="F3" s="31" t="s">
+      <c r="A3" s="40" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="41"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="42"/>
+      <c r="F3" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="26"/>
-      <c r="H3" s="32"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="47"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="28" t="s">
+      <c r="A4" s="43" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="29"/>
-      <c r="C4" s="29"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="30"/>
+      <c r="B4" s="44"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="44"/>
+      <c r="E4" s="45"/>
       <c r="F4" s="12" t="s">
         <v>5</v>
       </c>
@@ -1204,63 +1231,63 @@
       </c>
     </row>
     <row r="5" spans="1:43" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="43" t="s">
+      <c r="A5" s="37" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" s="38"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="38"/>
+      <c r="E5" s="38"/>
+      <c r="F5" s="38"/>
+      <c r="G5" s="38"/>
+      <c r="H5" s="39"/>
+    </row>
+    <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="44"/>
-      <c r="C5" s="44"/>
-      <c r="D5" s="44"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="44"/>
-      <c r="G5" s="44"/>
-      <c r="H5" s="45"/>
-    </row>
-    <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="33" t="s">
+      <c r="B6" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="41" t="s">
+      <c r="C6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="D6" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="E6" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="F6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="G6" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="H6" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="H6" s="7" t="s">
+    </row>
+    <row r="7" spans="1:43" s="2" customFormat="1" ht="324.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="27"/>
+      <c r="B7" s="36"/>
+      <c r="C7" s="20" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="7" spans="1:43" s="2" customFormat="1" ht="324.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="34"/>
-      <c r="B7" s="42"/>
-      <c r="C7" s="20" t="s">
+      <c r="D7" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="20" t="s">
+      <c r="E7" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="E7" s="20" t="s">
+      <c r="F7" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="F7" s="20" t="s">
+      <c r="G7" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="G7" s="20" t="s">
+      <c r="H7" s="21" t="s">
         <v>21</v>
-      </c>
-      <c r="H7" s="21" t="s">
-        <v>22</v>
       </c>
       <c r="I7"/>
       <c r="J7"/>
@@ -1299,16 +1326,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A8" s="35" t="s">
-        <v>23</v>
-      </c>
-      <c r="B8" s="36"/>
-      <c r="C8" s="36"/>
-      <c r="D8" s="36"/>
-      <c r="E8" s="36"/>
-      <c r="F8" s="36"/>
-      <c r="G8" s="36"/>
-      <c r="H8" s="37"/>
+      <c r="A8" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="30"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="31"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1347,17 +1374,17 @@
     </row>
     <row r="9" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="B9" s="22">
-        <v>45579</v>
+        <v>26</v>
+      </c>
+      <c r="B9" s="49" t="s">
+        <v>44</v>
       </c>
       <c r="C9" s="14"/>
       <c r="D9" s="15"/>
       <c r="E9" s="15"/>
       <c r="F9" s="15"/>
       <c r="G9" s="15"/>
-      <c r="H9" s="47"/>
+      <c r="H9" s="24"/>
       <c r="I9"/>
       <c r="J9"/>
       <c r="K9"/>
@@ -1396,16 +1423,18 @@
     </row>
     <row r="10" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="B10" s="8"/>
-      <c r="C10" s="46"/>
+        <v>28</v>
+      </c>
+      <c r="B10" s="48">
+        <v>45728</v>
+      </c>
+      <c r="C10" s="23"/>
       <c r="D10" s="15"/>
       <c r="E10" s="15"/>
       <c r="F10" s="15"/>
-      <c r="G10" s="46"/>
+      <c r="G10" s="23"/>
       <c r="H10" s="16"/>
-      <c r="I10" s="23"/>
+      <c r="I10" s="22"/>
       <c r="J10"/>
       <c r="K10"/>
       <c r="L10"/>
@@ -1443,13 +1472,16 @@
     </row>
     <row r="11" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="C11" s="46"/>
-      <c r="D11" s="46"/>
+        <v>27</v>
+      </c>
+      <c r="B11" s="50">
+        <v>45642</v>
+      </c>
+      <c r="C11" s="23"/>
+      <c r="D11" s="23"/>
       <c r="E11" s="15"/>
-      <c r="F11" s="46"/>
-      <c r="G11" s="46"/>
+      <c r="F11" s="23"/>
+      <c r="G11" s="23"/>
       <c r="H11" s="16"/>
       <c r="I11"/>
       <c r="J11"/>
@@ -1489,14 +1521,16 @@
     </row>
     <row r="12" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="B12" s="8"/>
-      <c r="C12" s="46"/>
+        <v>34</v>
+      </c>
+      <c r="B12" s="51">
+        <v>45966</v>
+      </c>
+      <c r="C12" s="23"/>
       <c r="D12" s="15"/>
       <c r="E12" s="15"/>
       <c r="F12" s="15"/>
-      <c r="G12" s="46"/>
+      <c r="G12" s="23"/>
       <c r="H12" s="16"/>
       <c r="I12"/>
       <c r="J12"/>
@@ -1536,14 +1570,16 @@
     </row>
     <row r="13" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="B13" s="8"/>
-      <c r="C13" s="46"/>
+        <v>36</v>
+      </c>
+      <c r="B13" s="51">
+        <v>46002</v>
+      </c>
+      <c r="C13" s="23"/>
       <c r="D13" s="15"/>
       <c r="E13" s="15"/>
-      <c r="F13" s="46"/>
-      <c r="G13" s="46"/>
+      <c r="F13" s="23"/>
+      <c r="G13" s="23"/>
       <c r="H13" s="16"/>
       <c r="I13"/>
       <c r="J13"/>
@@ -1583,14 +1619,16 @@
     </row>
     <row r="14" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="B14" s="8"/>
-      <c r="C14" s="46"/>
+        <v>35</v>
+      </c>
+      <c r="B14" s="51">
+        <v>46073</v>
+      </c>
+      <c r="C14" s="23"/>
       <c r="D14" s="15"/>
       <c r="E14" s="15"/>
       <c r="F14" s="15"/>
-      <c r="G14" s="46"/>
+      <c r="G14" s="23"/>
       <c r="H14" s="16"/>
       <c r="I14"/>
       <c r="J14"/>
@@ -1630,14 +1668,16 @@
     </row>
     <row r="15" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="B15" s="8"/>
-      <c r="C15" s="46"/>
+        <v>37</v>
+      </c>
+      <c r="B15" s="51">
+        <v>46025</v>
+      </c>
+      <c r="C15" s="23"/>
       <c r="D15" s="15"/>
       <c r="E15" s="15"/>
       <c r="F15" s="15"/>
-      <c r="G15" s="46"/>
+      <c r="G15" s="23"/>
       <c r="H15" s="16"/>
       <c r="I15"/>
       <c r="J15"/>
@@ -1677,14 +1717,16 @@
     </row>
     <row r="16" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="B16" s="8"/>
-      <c r="C16" s="46"/>
+        <v>40</v>
+      </c>
+      <c r="B16" s="51">
+        <v>45777</v>
+      </c>
+      <c r="C16" s="23"/>
       <c r="D16" s="15"/>
       <c r="E16" s="15"/>
       <c r="F16" s="15"/>
-      <c r="G16" s="46"/>
+      <c r="G16" s="23"/>
       <c r="H16" s="16"/>
       <c r="I16"/>
       <c r="J16"/>
@@ -1813,16 +1855,16 @@
       <c r="AQ18"/>
     </row>
     <row r="19" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A19" s="38" t="s">
-        <v>24</v>
-      </c>
-      <c r="B19" s="39"/>
-      <c r="C19" s="39"/>
-      <c r="D19" s="39"/>
-      <c r="E19" s="39"/>
-      <c r="F19" s="39"/>
-      <c r="G19" s="39"/>
-      <c r="H19" s="40"/>
+      <c r="A19" s="32" t="s">
+        <v>23</v>
+      </c>
+      <c r="B19" s="33"/>
+      <c r="C19" s="33"/>
+      <c r="D19" s="33"/>
+      <c r="E19" s="33"/>
+      <c r="F19" s="33"/>
+      <c r="G19" s="33"/>
+      <c r="H19" s="34"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1861,14 +1903,16 @@
     </row>
     <row r="20" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="B20" s="8"/>
-      <c r="C20" s="46"/>
-      <c r="D20" s="46"/>
+        <v>41</v>
+      </c>
+      <c r="B20" s="52" t="s">
+        <v>44</v>
+      </c>
+      <c r="C20" s="23"/>
+      <c r="D20" s="23"/>
       <c r="E20" s="15"/>
       <c r="F20" s="15"/>
-      <c r="G20" s="46"/>
+      <c r="G20" s="23"/>
       <c r="H20" s="16"/>
       <c r="I20"/>
       <c r="J20"/>
@@ -1908,14 +1952,16 @@
     </row>
     <row r="21" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="B21" s="8"/>
-      <c r="C21" s="46"/>
+        <v>32</v>
+      </c>
+      <c r="B21" s="52" t="s">
+        <v>44</v>
+      </c>
+      <c r="C21" s="23"/>
       <c r="D21" s="15"/>
       <c r="E21" s="15"/>
-      <c r="F21" s="46"/>
-      <c r="G21" s="46"/>
+      <c r="F21" s="23"/>
+      <c r="G21" s="23"/>
       <c r="H21" s="16"/>
       <c r="I21"/>
       <c r="J21"/>
@@ -1955,13 +2001,15 @@
     </row>
     <row r="22" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B22" s="8"/>
-      <c r="C22" s="46"/>
+        <v>31</v>
+      </c>
+      <c r="B22" s="52" t="s">
+        <v>44</v>
+      </c>
+      <c r="C22" s="23"/>
       <c r="D22" s="15"/>
       <c r="E22" s="15"/>
-      <c r="F22" s="46"/>
+      <c r="F22" s="23"/>
       <c r="G22" s="15"/>
       <c r="H22" s="16"/>
       <c r="I22"/>
@@ -2002,11 +2050,13 @@
     </row>
     <row r="23" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="B23" s="8"/>
-      <c r="C23" s="46"/>
-      <c r="D23" s="46"/>
+        <v>39</v>
+      </c>
+      <c r="B23" s="51">
+        <v>45785</v>
+      </c>
+      <c r="C23" s="23"/>
+      <c r="D23" s="23"/>
       <c r="E23" s="15"/>
       <c r="F23" s="15"/>
       <c r="G23" s="15"/>
@@ -2183,16 +2233,16 @@
       <c r="AQ26"/>
     </row>
     <row r="27" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A27" s="38" t="s">
-        <v>25</v>
-      </c>
-      <c r="B27" s="39"/>
-      <c r="C27" s="39"/>
-      <c r="D27" s="39"/>
-      <c r="E27" s="39"/>
-      <c r="F27" s="39"/>
-      <c r="G27" s="39"/>
-      <c r="H27" s="40"/>
+      <c r="A27" s="32" t="s">
+        <v>24</v>
+      </c>
+      <c r="B27" s="33"/>
+      <c r="C27" s="33"/>
+      <c r="D27" s="33"/>
+      <c r="E27" s="33"/>
+      <c r="F27" s="33"/>
+      <c r="G27" s="33"/>
+      <c r="H27" s="34"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2231,14 +2281,16 @@
     </row>
     <row r="28" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="B28" s="8"/>
-      <c r="C28" s="46"/>
-      <c r="D28" s="46"/>
+        <v>41</v>
+      </c>
+      <c r="B28" s="52" t="s">
+        <v>44</v>
+      </c>
+      <c r="C28" s="23"/>
+      <c r="D28" s="23"/>
       <c r="E28" s="15"/>
       <c r="F28" s="15"/>
-      <c r="G28" s="46"/>
+      <c r="G28" s="23"/>
       <c r="H28" s="16"/>
       <c r="I28"/>
       <c r="J28"/>
@@ -2278,14 +2330,16 @@
     </row>
     <row r="29" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="B29" s="8"/>
-      <c r="C29" s="46"/>
-      <c r="D29" s="46"/>
+        <v>29</v>
+      </c>
+      <c r="B29" s="52" t="s">
+        <v>45</v>
+      </c>
+      <c r="C29" s="23"/>
+      <c r="D29" s="23"/>
       <c r="E29" s="15"/>
-      <c r="F29" s="46"/>
-      <c r="G29" s="46"/>
+      <c r="F29" s="23"/>
+      <c r="G29" s="23"/>
       <c r="H29" s="16"/>
       <c r="I29"/>
       <c r="J29"/>
@@ -2325,15 +2379,17 @@
     </row>
     <row r="30" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B30" s="8"/>
+        <v>30</v>
+      </c>
+      <c r="B30" s="53">
+        <v>45658</v>
+      </c>
       <c r="C30" s="15"/>
       <c r="D30" s="15"/>
-      <c r="E30" s="46"/>
-      <c r="F30" s="46"/>
-      <c r="G30" s="46"/>
-      <c r="H30" s="47"/>
+      <c r="E30" s="23"/>
+      <c r="F30" s="23"/>
+      <c r="G30" s="23"/>
+      <c r="H30" s="24"/>
       <c r="I30"/>
       <c r="J30"/>
       <c r="K30"/>
@@ -2372,14 +2428,16 @@
     </row>
     <row r="31" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="B31" s="8"/>
-      <c r="C31" s="46"/>
+        <v>33</v>
+      </c>
+      <c r="B31" s="53">
+        <v>45992</v>
+      </c>
+      <c r="C31" s="23"/>
       <c r="D31" s="15"/>
       <c r="E31" s="15"/>
-      <c r="F31" s="46"/>
-      <c r="G31" s="46"/>
+      <c r="F31" s="23"/>
+      <c r="G31" s="23"/>
       <c r="H31" s="16"/>
       <c r="I31"/>
       <c r="J31"/>
@@ -2419,15 +2477,17 @@
     </row>
     <row r="32" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="B32" s="8"/>
+        <v>38</v>
+      </c>
+      <c r="B32" s="53">
+        <v>45992</v>
+      </c>
       <c r="C32" s="15"/>
-      <c r="D32" s="46"/>
+      <c r="D32" s="23"/>
       <c r="E32" s="15"/>
       <c r="F32" s="15"/>
       <c r="G32" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H32" s="16"/>
       <c r="I32"/>
@@ -2469,11 +2529,11 @@
     <row r="33" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="9"/>
       <c r="B33" s="8"/>
-      <c r="C33" s="48"/>
-      <c r="D33" s="48"/>
+      <c r="C33" s="25"/>
+      <c r="D33" s="25"/>
       <c r="E33" s="15"/>
-      <c r="F33" s="48"/>
-      <c r="G33" s="48"/>
+      <c r="F33" s="25"/>
+      <c r="G33" s="25"/>
       <c r="H33" s="16"/>
       <c r="I33"/>
       <c r="J33"/>
@@ -2649,6 +2709,11 @@
     <row r="81" customFormat="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -2656,11 +2721,6 @@
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -2671,26 +2731,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="78b7d894-c7e3-470e-a432-745d16620d5f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="aef17354-bb95-43df-ae29-2de24b17c318" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100225CB4ADA382224D88C6043966D844BA" ma:contentTypeVersion="12" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="73a2b8ae3b91ced84031e25ba38c8442">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="78b7d894-c7e3-470e-a432-745d16620d5f" xmlns:ns3="aef17354-bb95-43df-ae29-2de24b17c318" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fdc26ae3f96df8659fd11315e8834360" ns2:_="" ns3:_="">
     <xsd:import namespace="78b7d894-c7e3-470e-a432-745d16620d5f"/>
@@ -2891,26 +2931,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2D1CAE4-71AE-4724-BB88-512758980E7F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="78b7d894-c7e3-470e-a432-745d16620d5f"/>
-    <ds:schemaRef ds:uri="aef17354-bb95-43df-ae29-2de24b17c318"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8A372A1D-F884-4120-AE10-3A1D047E2D07}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="78b7d894-c7e3-470e-a432-745d16620d5f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="aef17354-bb95-43df-ae29-2de24b17c318" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D18C4935-D199-415A-A1F7-6863E4383E64}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2927,4 +2968,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8A372A1D-F884-4120-AE10-3A1D047E2D07}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2D1CAE4-71AE-4724-BB88-512758980E7F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="78b7d894-c7e3-470e-a432-745d16620d5f"/>
+    <ds:schemaRef ds:uri="aef17354-bb95-43df-ae29-2de24b17c318"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update navbar link order and about section
</commit_message>
<xml_diff>
--- a/public/8 - ANNEXE VI.1 - EPREUVE E5 TABLEAU DE SYNTHESE - BTS SIO 2026 MOUHOUBI Noam.xlsx
+++ b/public/8 - ANNEXE VI.1 - EPREUVE E5 TABLEAU DE SYNTHESE - BTS SIO 2026 MOUHOUBI Noam.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\noamm\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nmouhoubi\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4440D4AD-8EE8-47A6-A57C-3FD715E3783D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BB7BBC4-817C-40C6-B24A-845FAF29E4C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E5" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="43">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -150,18 +150,12 @@
     <t>Migration Windows 11 de tous les postes utilisateurs</t>
   </si>
   <si>
-    <t>Développement d'une IA interne accessible depuis l'intranet</t>
-  </si>
-  <si>
     <t>Gestion de parc informatique</t>
   </si>
   <si>
     <t>Préparation de postes utilisateurs physique</t>
   </si>
   <si>
-    <t>Refonte complète du réseau internet</t>
-  </si>
-  <si>
     <t>Windows Server avec Active Directory</t>
   </si>
   <si>
@@ -184,9 +178,6 @@
   </si>
   <si>
     <t>Maintenance et support utilisateur via Easyvista</t>
-  </si>
-  <si>
-    <t>s</t>
   </si>
   <si>
     <t>Adresse URL du portfolio : https://nmouhoubi.com/</t>
@@ -692,7 +683,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -767,15 +758,57 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -809,47 +842,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1160,66 +1154,66 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AQ81"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="70.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.85546875" style="1" customWidth="1"/>
-    <col min="3" max="8" width="18.7109375" style="1" customWidth="1"/>
-    <col min="9" max="43" width="11.42578125" customWidth="1"/>
-    <col min="44" max="16384" width="10.85546875" style="1"/>
+    <col min="1" max="1" width="70.44140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="10.88671875" style="1" customWidth="1"/>
+    <col min="3" max="8" width="18.6640625" style="1" customWidth="1"/>
+    <col min="9" max="43" width="11.44140625" customWidth="1"/>
+    <col min="44" max="16384" width="10.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="28" t="s">
+    <row r="1" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28" t="s">
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="28"/>
-    </row>
-    <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="28" t="s">
+      <c r="H1" s="32"/>
+    </row>
+    <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-    </row>
-    <row r="3" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="40" t="s">
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+    </row>
+    <row r="3" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="41"/>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="42"/>
-      <c r="F3" s="46" t="s">
+      <c r="B3" s="34"/>
+      <c r="C3" s="34"/>
+      <c r="D3" s="34"/>
+      <c r="E3" s="35"/>
+      <c r="F3" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="41"/>
-      <c r="H3" s="47"/>
+      <c r="G3" s="34"/>
+      <c r="H3" s="40"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
-    <row r="4" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="43" t="s">
+    <row r="4" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="44"/>
-      <c r="C4" s="44"/>
-      <c r="D4" s="44"/>
-      <c r="E4" s="45"/>
+      <c r="B4" s="37"/>
+      <c r="C4" s="37"/>
+      <c r="D4" s="37"/>
+      <c r="E4" s="38"/>
       <c r="F4" s="12" t="s">
         <v>5</v>
       </c>
@@ -1230,23 +1224,23 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:43" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="37" t="s">
-        <v>43</v>
-      </c>
-      <c r="B5" s="38"/>
-      <c r="C5" s="38"/>
-      <c r="D5" s="38"/>
-      <c r="E5" s="38"/>
-      <c r="F5" s="38"/>
-      <c r="G5" s="38"/>
-      <c r="H5" s="39"/>
-    </row>
-    <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="26" t="s">
+    <row r="5" spans="1:43" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="51" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5" s="52"/>
+      <c r="C5" s="52"/>
+      <c r="D5" s="52"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="52"/>
+      <c r="G5" s="52"/>
+      <c r="H5" s="53"/>
+    </row>
+    <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="41" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="35" t="s">
+      <c r="B6" s="49" t="s">
         <v>9</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1268,9 +1262,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:43" s="2" customFormat="1" ht="324.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="27"/>
-      <c r="B7" s="36"/>
+    <row r="7" spans="1:43" s="2" customFormat="1" ht="324.89999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="42"/>
+      <c r="B7" s="50"/>
       <c r="C7" s="20" t="s">
         <v>16</v>
       </c>
@@ -1325,17 +1319,17 @@
       <c r="AP7"/>
       <c r="AQ7"/>
     </row>
-    <row r="8" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A8" s="29" t="s">
+    <row r="8" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A8" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="30"/>
-      <c r="C8" s="30"/>
-      <c r="D8" s="30"/>
-      <c r="E8" s="30"/>
-      <c r="F8" s="30"/>
-      <c r="G8" s="30"/>
-      <c r="H8" s="31"/>
+      <c r="B8" s="44"/>
+      <c r="C8" s="44"/>
+      <c r="D8" s="44"/>
+      <c r="E8" s="44"/>
+      <c r="F8" s="44"/>
+      <c r="G8" s="44"/>
+      <c r="H8" s="45"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1372,12 +1366,12 @@
       <c r="AP8"/>
       <c r="AQ8"/>
     </row>
-    <row r="9" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="B9" s="49" t="s">
-        <v>44</v>
+      <c r="B9" s="27" t="s">
+        <v>41</v>
       </c>
       <c r="C9" s="14"/>
       <c r="D9" s="15"/>
@@ -1421,11 +1415,11 @@
       <c r="AP9"/>
       <c r="AQ9"/>
     </row>
-    <row r="10" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="B10" s="48">
+      <c r="B10" s="26">
         <v>45728</v>
       </c>
       <c r="C10" s="23"/>
@@ -1470,11 +1464,11 @@
       <c r="AP10"/>
       <c r="AQ10"/>
     </row>
-    <row r="11" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="B11" s="50">
+      <c r="B11" s="28">
         <v>45642</v>
       </c>
       <c r="C11" s="23"/>
@@ -1519,11 +1513,11 @@
       <c r="AP11"/>
       <c r="AQ11"/>
     </row>
-    <row r="12" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="B12" s="51">
+        <v>32</v>
+      </c>
+      <c r="B12" s="29">
         <v>45966</v>
       </c>
       <c r="C12" s="23"/>
@@ -1568,11 +1562,11 @@
       <c r="AP12"/>
       <c r="AQ12"/>
     </row>
-    <row r="13" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="B13" s="51">
+        <v>34</v>
+      </c>
+      <c r="B13" s="29">
         <v>46002</v>
       </c>
       <c r="C13" s="23"/>
@@ -1617,11 +1611,11 @@
       <c r="AP13"/>
       <c r="AQ13"/>
     </row>
-    <row r="14" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="B14" s="51">
+        <v>33</v>
+      </c>
+      <c r="B14" s="29">
         <v>46073</v>
       </c>
       <c r="C14" s="23"/>
@@ -1666,11 +1660,11 @@
       <c r="AP14"/>
       <c r="AQ14"/>
     </row>
-    <row r="15" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="B15" s="51">
+        <v>35</v>
+      </c>
+      <c r="B15" s="29">
         <v>46025</v>
       </c>
       <c r="C15" s="23"/>
@@ -1715,11 +1709,11 @@
       <c r="AP15"/>
       <c r="AQ15"/>
     </row>
-    <row r="16" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="B16" s="51">
+        <v>38</v>
+      </c>
+      <c r="B16" s="29">
         <v>45777</v>
       </c>
       <c r="C16" s="23"/>
@@ -1764,7 +1758,7 @@
       <c r="AP16"/>
       <c r="AQ16"/>
     </row>
-    <row r="17" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="9"/>
       <c r="B17" s="8"/>
       <c r="C17" s="15"/>
@@ -1809,7 +1803,7 @@
       <c r="AP17"/>
       <c r="AQ17"/>
     </row>
-    <row r="18" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="9"/>
       <c r="B18" s="8"/>
       <c r="C18" s="15"/>
@@ -1854,17 +1848,17 @@
       <c r="AP18"/>
       <c r="AQ18"/>
     </row>
-    <row r="19" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A19" s="32" t="s">
+    <row r="19" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A19" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="B19" s="33"/>
-      <c r="C19" s="33"/>
-      <c r="D19" s="33"/>
-      <c r="E19" s="33"/>
-      <c r="F19" s="33"/>
-      <c r="G19" s="33"/>
-      <c r="H19" s="34"/>
+      <c r="B19" s="47"/>
+      <c r="C19" s="47"/>
+      <c r="D19" s="47"/>
+      <c r="E19" s="47"/>
+      <c r="F19" s="47"/>
+      <c r="G19" s="47"/>
+      <c r="H19" s="48"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1901,12 +1895,12 @@
       <c r="AP19"/>
       <c r="AQ19"/>
     </row>
-    <row r="20" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B20" s="30" t="s">
         <v>41</v>
-      </c>
-      <c r="B20" s="52" t="s">
-        <v>44</v>
       </c>
       <c r="C20" s="23"/>
       <c r="D20" s="23"/>
@@ -1950,12 +1944,12 @@
       <c r="AP20"/>
       <c r="AQ20"/>
     </row>
-    <row r="21" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B21" s="52" t="s">
-        <v>44</v>
+        <v>31</v>
+      </c>
+      <c r="B21" s="30" t="s">
+        <v>41</v>
       </c>
       <c r="C21" s="23"/>
       <c r="D21" s="15"/>
@@ -1999,12 +1993,12 @@
       <c r="AP21"/>
       <c r="AQ21"/>
     </row>
-    <row r="22" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B22" s="52" t="s">
-        <v>44</v>
+        <v>30</v>
+      </c>
+      <c r="B22" s="30" t="s">
+        <v>41</v>
       </c>
       <c r="C22" s="23"/>
       <c r="D22" s="15"/>
@@ -2048,11 +2042,11 @@
       <c r="AP22"/>
       <c r="AQ22"/>
     </row>
-    <row r="23" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="B23" s="51">
+        <v>37</v>
+      </c>
+      <c r="B23" s="29">
         <v>45785</v>
       </c>
       <c r="C23" s="23"/>
@@ -2097,7 +2091,7 @@
       <c r="AP23"/>
       <c r="AQ23"/>
     </row>
-    <row r="24" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="9"/>
       <c r="B24" s="8"/>
       <c r="C24" s="15"/>
@@ -2142,7 +2136,7 @@
       <c r="AP24"/>
       <c r="AQ24"/>
     </row>
-    <row r="25" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="9"/>
       <c r="B25" s="8"/>
       <c r="C25" s="15"/>
@@ -2187,7 +2181,7 @@
       <c r="AP25"/>
       <c r="AQ25"/>
     </row>
-    <row r="26" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="9"/>
       <c r="B26" s="8"/>
       <c r="C26" s="15"/>
@@ -2232,17 +2226,17 @@
       <c r="AP26"/>
       <c r="AQ26"/>
     </row>
-    <row r="27" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A27" s="32" t="s">
+    <row r="27" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A27" s="46" t="s">
         <v>24</v>
       </c>
-      <c r="B27" s="33"/>
-      <c r="C27" s="33"/>
-      <c r="D27" s="33"/>
-      <c r="E27" s="33"/>
-      <c r="F27" s="33"/>
-      <c r="G27" s="33"/>
-      <c r="H27" s="34"/>
+      <c r="B27" s="47"/>
+      <c r="C27" s="47"/>
+      <c r="D27" s="47"/>
+      <c r="E27" s="47"/>
+      <c r="F27" s="47"/>
+      <c r="G27" s="47"/>
+      <c r="H27" s="48"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2279,12 +2273,12 @@
       <c r="AP27"/>
       <c r="AQ27"/>
     </row>
-    <row r="28" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B28" s="30" t="s">
         <v>41</v>
-      </c>
-      <c r="B28" s="52" t="s">
-        <v>44</v>
       </c>
       <c r="C28" s="23"/>
       <c r="D28" s="23"/>
@@ -2328,12 +2322,12 @@
       <c r="AP28"/>
       <c r="AQ28"/>
     </row>
-    <row r="29" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="B29" s="52" t="s">
-        <v>45</v>
+      <c r="B29" s="30" t="s">
+        <v>42</v>
       </c>
       <c r="C29" s="23"/>
       <c r="D29" s="23"/>
@@ -2377,19 +2371,19 @@
       <c r="AP29"/>
       <c r="AQ29"/>
     </row>
-    <row r="30" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="B30" s="53">
+        <v>36</v>
+      </c>
+      <c r="B30" s="31">
         <v>45658</v>
       </c>
       <c r="C30" s="15"/>
-      <c r="D30" s="15"/>
-      <c r="E30" s="23"/>
-      <c r="F30" s="23"/>
-      <c r="G30" s="23"/>
-      <c r="H30" s="24"/>
+      <c r="D30" s="23"/>
+      <c r="E30" s="25"/>
+      <c r="F30" s="25"/>
+      <c r="G30" s="25"/>
+      <c r="H30" s="54"/>
       <c r="I30"/>
       <c r="J30"/>
       <c r="K30"/>
@@ -2426,18 +2420,14 @@
       <c r="AP30"/>
       <c r="AQ30"/>
     </row>
-    <row r="31" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="B31" s="53">
-        <v>45992</v>
-      </c>
-      <c r="C31" s="23"/>
+    <row r="31" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="9"/>
+      <c r="B31" s="31"/>
+      <c r="C31" s="25"/>
       <c r="D31" s="15"/>
       <c r="E31" s="15"/>
-      <c r="F31" s="23"/>
-      <c r="G31" s="23"/>
+      <c r="F31" s="25"/>
+      <c r="G31" s="25"/>
       <c r="H31" s="16"/>
       <c r="I31"/>
       <c r="J31"/>
@@ -2475,20 +2465,14 @@
       <c r="AP31"/>
       <c r="AQ31"/>
     </row>
-    <row r="32" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="B32" s="53">
-        <v>45992</v>
-      </c>
+    <row r="32" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="9"/>
+      <c r="B32" s="31"/>
       <c r="C32" s="15"/>
-      <c r="D32" s="23"/>
+      <c r="D32" s="25"/>
       <c r="E32" s="15"/>
       <c r="F32" s="15"/>
-      <c r="G32" s="15" t="s">
-        <v>42</v>
-      </c>
+      <c r="G32" s="15"/>
       <c r="H32" s="16"/>
       <c r="I32"/>
       <c r="J32"/>
@@ -2526,7 +2510,7 @@
       <c r="AP32"/>
       <c r="AQ32"/>
     </row>
-    <row r="33" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="9"/>
       <c r="B33" s="8"/>
       <c r="C33" s="25"/>
@@ -2571,7 +2555,7 @@
       <c r="AP33"/>
       <c r="AQ33"/>
     </row>
-    <row r="34" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="10"/>
       <c r="B34" s="11"/>
       <c r="C34" s="17"/>
@@ -2616,7 +2600,7 @@
       <c r="AP34"/>
       <c r="AQ34"/>
     </row>
-    <row r="35" spans="1:43" s="2" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:43" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A35" s="5"/>
       <c r="B35" s="3"/>
       <c r="C35" s="4"/>
@@ -2661,59 +2645,54 @@
       <c r="AP35"/>
       <c r="AQ35"/>
     </row>
-    <row r="36" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="37" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="38" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="39" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="40" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="41" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="42" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="43" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="44" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="45" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="46" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="47" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="48" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="49" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="50" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="51" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="52" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="53" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="54" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="55" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="56" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="57" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="58" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="59" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="60" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="61" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="62" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="63" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="64" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="65" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="66" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="67" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="68" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="69" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="70" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="71" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="72" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="73" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="74" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="75" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="76" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="77" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="78" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="79" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="80" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="81" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="36" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="37" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="40" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="42" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="43" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="45" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="46" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="47" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="48" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="49" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="50" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="51" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="52" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="53" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="54" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="55" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="56" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="57" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="58" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="59" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="60" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="61" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="62" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="63" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="64" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="65" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="66" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="67" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="68" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="69" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="70" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="71" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="72" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="73" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="74" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="75" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="76" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="77" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="78" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="79" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="80" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="81" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -2721,6 +2700,11 @@
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -2932,15 +2916,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="78b7d894-c7e3-470e-a432-745d16620d5f">
@@ -2949,6 +2924,15 @@
     <TaxCatchAll xmlns="aef17354-bb95-43df-ae29-2de24b17c318" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2971,14 +2955,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8A372A1D-F884-4120-AE10-3A1D047E2D07}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2D1CAE4-71AE-4724-BB88-512758980E7F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -2987,4 +2963,12 @@
     <ds:schemaRef ds:uri="aef17354-bb95-43df-ae29-2de24b17c318"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8A372A1D-F884-4120-AE10-3A1D047E2D07}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>